<commit_message>
DOCS: updated SliderNew demo to show use of keyboard control
</commit_message>
<xml_diff>
--- a/psychopy/demos/builder/ratingsNew/fruitConditions.xlsx
+++ b/psychopy/demos/builder/ratingsNew/fruitConditions.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10513"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lpzjwp/code/psychopy/git/psychopy/demos/builder/ratingsNew/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lpzjwp\code\psychopy\git\psychopy\demos\builder\ratingsNew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{47E87EE8-1B66-6A40-8CF5-653723B825DB}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11580" yWindow="5460" windowWidth="28040" windowHeight="17440" xr2:uid="{93372140-D705-D744-8D56-065E329B1ACF}"/>
+    <workbookView xWindow="11580" yWindow="5460" windowWidth="28035" windowHeight="17445"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>apple</t>
   </si>
@@ -36,16 +35,13 @@
     <t>banana</t>
   </si>
   <si>
-    <t>satsuma</t>
-  </si>
-  <si>
     <t>fruitName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -399,33 +395,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D88FB63-1422-CA48-A22E-C82383F14D65}">
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>